<commit_message>
fixed excel order update and tables in admin driver greeter school
</commit_message>
<xml_diff>
--- a/backend/templates/student_upload_template.xlsx
+++ b/backend/templates/student_upload_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Students" sheetId="1" r:id="rId1"/>
+    <sheet name="Student Upload Template" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,26 +397,45 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:Q6"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="6.83203125" customWidth="1"/>
+    <col min="5" max="5" width="8.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+    <col min="13" max="13" width="15.83203125" customWidth="1"/>
+    <col min="14" max="14" width="25.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="12.83203125" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Trip #</v>
+        <v>Trip</v>
       </c>
       <c r="B1" t="str">
-        <v>Actual Arrival Time / Departure Pick Up Time</v>
+        <v>Arr Time</v>
       </c>
       <c r="C1" t="str">
-        <v>Arr Time / Dep PU</v>
+        <v>Flight #</v>
       </c>
       <c r="D1" t="str">
-        <v>Flight #</v>
+        <v>D/I</v>
       </c>
       <c r="E1" t="str">
-        <v>I or M / F</v>
+        <v>M or F</v>
       </c>
       <c r="F1" t="str">
-        <v>Student Number</v>
+        <v>Student Numb</v>
       </c>
       <c r="G1" t="str">
         <v>Student Given Name</v>
@@ -431,7 +450,7 @@
         <v>Host Family Name</v>
       </c>
       <c r="K1" t="str">
-        <v>Phone H=Home C=Cell B=Business</v>
+        <v>Phone</v>
       </c>
       <c r="L1" t="str">
         <v>Address</v>
@@ -443,15 +462,12 @@
         <v>Special Instructions</v>
       </c>
       <c r="O1" t="str">
-        <v>Study Permit Y or N</v>
+        <v>Study Permit Y/N</v>
       </c>
       <c r="P1" t="str">
         <v>School</v>
       </c>
       <c r="Q1" t="str">
-        <v>Staff Member Assigned</v>
-      </c>
-      <c r="R1" t="str">
         <v>Client</v>
       </c>
     </row>
@@ -460,60 +476,269 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>2:00 AM / 6:00 AM</v>
+        <v>5:10 PM</v>
       </c>
       <c r="C2" t="str">
-        <v>2:00 AM / 6:00 AM</v>
+        <v>TK 075</v>
       </c>
       <c r="D2" t="str">
+        <v>I</v>
+      </c>
+      <c r="E2" t="str">
+        <v>M</v>
+      </c>
+      <c r="F2" t="str">
+        <v>733382</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Osama</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Alansar</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Rose</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Pugosa</v>
+      </c>
+      <c r="K2" t="str">
+        <v>C=6044909182</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Clinton Street</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Burnaby</v>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v>N</v>
+      </c>
+      <c r="P2" t="str">
+        <v>EC</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>EC</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>4:15 AM</v>
+      </c>
+      <c r="C3" t="str">
+        <v>AM 695</v>
+      </c>
+      <c r="D3" t="str">
+        <v>I</v>
+      </c>
+      <c r="E3" t="str">
+        <v>F</v>
+      </c>
+      <c r="F3" t="str">
+        <v>704047</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Judith</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Marcondes Armando</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Maria</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Santos</v>
+      </c>
+      <c r="K3" t="str">
+        <v>H=6041234567</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Main Street</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Vancouver</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Departs @ 8:15 AM</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="P3" t="str">
+        <v>ILSC</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>ILSC</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2:00 AM</v>
+      </c>
+      <c r="C4" t="str">
         <v>AS 6047</v>
       </c>
-      <c r="E2" t="str">
+      <c r="D4" t="str">
+        <v>I</v>
+      </c>
+      <c r="E4" t="str">
         <v>F</v>
       </c>
-      <c r="F2" t="str">
+      <c r="F4" t="str">
         <v>VE158887</v>
       </c>
-      <c r="G2" t="str">
+      <c r="G4" t="str">
         <v>Mariana</v>
       </c>
-      <c r="H2" t="str">
+      <c r="H4" t="str">
         <v>Palmieri Panazzolo</v>
       </c>
-      <c r="I2" t="str">
+      <c r="I4" t="str">
         <v>Angelica</v>
       </c>
-      <c r="J2" t="str">
+      <c r="J4" t="str">
         <v>Lim</v>
       </c>
-      <c r="K2" t="str">
-        <v>7782510236</v>
-      </c>
-      <c r="L2" t="str">
-        <v>6962 Fleming St</v>
-      </c>
-      <c r="M2" t="str">
+      <c r="K4" t="str">
+        <v>C=7782510236</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Fleming Street</v>
+      </c>
+      <c r="M4" t="str">
         <v>Vancouver</v>
       </c>
-      <c r="N2" t="str">
-        <v>Departs @ 6:00 AM</v>
-      </c>
-      <c r="O2" t="str">
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
         <v>Y</v>
       </c>
-      <c r="P2" t="str">
-        <v>ILSC</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>Jaskirat 1st Job</v>
-      </c>
-      <c r="R2" t="str">
-        <v>ILSC</v>
+      <c r="P4" t="str">
+        <v>VEC</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>VEC</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>6:30 PM</v>
+      </c>
+      <c r="C5" t="str">
+        <v>AC 123</v>
+      </c>
+      <c r="D5" t="str">
+        <v>D</v>
+      </c>
+      <c r="E5" t="str">
+        <v>M</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>John</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Smith</v>
+      </c>
+      <c r="I5" t="str">
+        <v>David</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Johnson</v>
+      </c>
+      <c r="K5" t="str">
+        <v>B=6049876543</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Oak Street</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Richmond</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Early pickup required</v>
+      </c>
+      <c r="O5" t="str">
+        <v>N</v>
+      </c>
+      <c r="P5" t="str">
+        <v>ILAC</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>ILAC</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>3:45 AM</v>
+      </c>
+      <c r="C6" t="str">
+        <v>WF 456</v>
+      </c>
+      <c r="D6" t="str">
+        <v>I</v>
+      </c>
+      <c r="E6" t="str">
+        <v>F</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>Sarah</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Williams</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Lisa</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Brown</v>
+      </c>
+      <c r="K6" t="str">
+        <v>H=7781234567</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Granville Street</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Vancouver</v>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v>Y</v>
+      </c>
+      <c r="P6" t="str">
+        <v>EC</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>EC</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>